<commit_message>
Actualizacion de paths para la pagina de Info casas
</commit_message>
<xml_diff>
--- a/remax_2/driver/Pass.xlsx
+++ b/remax_2/driver/Pass.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prueba\Desktop\Py\remax_2\driver\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matia\Desktop\RemaxCentury\BotRemax-main\remax_2\driver\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B289A418-AFF5-4A76-A19F-97D0364AA549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Infocasas" sheetId="2" r:id="rId1"/>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="50">
   <si>
     <t>Correo</t>
   </si>
@@ -96,9 +97,6 @@
   </si>
   <si>
     <t>Tel</t>
-  </si>
-  <si>
-    <t>alexavillamayorremax@gmail.com</t>
   </si>
   <si>
     <t>Cantidad Publicar</t>
@@ -478,9 +476,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>Benjavilla1991</t>
-  </si>
-  <si>
     <t>gisellremax@gmail.com</t>
   </si>
   <si>
@@ -496,27 +491,9 @@
     <t>Luisremax</t>
   </si>
   <si>
-    <t>Valeriacuevasremax@gmail.com</t>
-  </si>
-  <si>
-    <t>VALERIAREMAX</t>
-  </si>
-  <si>
     <t xml:space="preserve">0972466885 </t>
   </si>
   <si>
-    <t>Charly901210</t>
-  </si>
-  <si>
-    <t>gdelgado995@gmail.com</t>
-  </si>
-  <si>
-    <t>2205ambar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0961713273 </t>
-  </si>
-  <si>
     <t>valeriacuevasremax@gmail.com</t>
   </si>
   <si>
@@ -526,12 +503,6 @@
     <t>Margaremax</t>
   </si>
   <si>
-    <t>maggygodelafs84@gmail.com</t>
-  </si>
-  <si>
-    <t>Marga204</t>
-  </si>
-  <si>
     <t>ftp</t>
   </si>
   <si>
@@ -544,17 +515,17 @@
     <t>Keilagaleanoremax@gmail.com</t>
   </si>
   <si>
-    <t>keilaremax</t>
-  </si>
-  <si>
     <t>0971521781</t>
+  </si>
+  <si>
+    <t>c21novaasesorale@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="13" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -651,6 +622,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -724,7 +703,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
@@ -776,7 +755,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1097,7 +1083,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1125,13 +1111,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>36</v>
+        <v>49</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>16</v>
@@ -1142,16 +1128,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1159,13 +1145,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>18</v>
@@ -1176,16 +1162,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C5" s="3">
         <v>12345678</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1193,16 +1179,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -1210,21 +1196,21 @@
         <v>6</v>
       </c>
       <c r="B7" s="22" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="C7" s="23">
         <v>12345678</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>20</v>
@@ -1232,17 +1218,17 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1"/>
-    <hyperlink ref="B4" r:id="rId2"/>
-    <hyperlink ref="B6" r:id="rId3"/>
-    <hyperlink ref="B7" r:id="rId4"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="B6" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="B7" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1274,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>16</v>
@@ -1291,7 +1277,7 @@
         <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E3" s="11" t="s">
         <v>17</v>
@@ -1308,7 +1294,7 @@
         <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>18</v>
@@ -1325,7 +1311,7 @@
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>19</v>
@@ -1342,20 +1328,20 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C1"/>
+  <autoFilter ref="A1:C1" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1"/>
-    <hyperlink ref="B2" r:id="rId2"/>
-    <hyperlink ref="B3" r:id="rId3"/>
-    <hyperlink ref="B5" r:id="rId4"/>
-    <hyperlink ref="B4" r:id="rId5"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B2" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="B3" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="B4" r:id="rId5" xr:uid="{00000000-0004-0000-0100-000004000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
@@ -1363,8 +1349,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" bestFit="1" customWidth="1"/>
@@ -1394,7 +1380,7 @@
         <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>16</v>
@@ -1404,102 +1390,55 @@
       <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>48</v>
-      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="5"/>
+      <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>18</v>
-      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="3"/>
+      <c r="E4" s="11"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="20">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="11" t="s">
-        <v>44</v>
-      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="3"/>
+      <c r="E5" s="11"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="20">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>55</v>
-      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="5"/>
+      <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="25">
         <v>6</v>
       </c>
-      <c r="B7" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>59</v>
-      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="24"/>
+      <c r="E7" s="11"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E8" s="26"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1"/>
-    <hyperlink ref="B3" r:id="rId2"/>
-    <hyperlink ref="B4" r:id="rId3"/>
-    <hyperlink ref="B5" r:id="rId4"/>
-    <hyperlink ref="B6" r:id="rId5"/>
-    <hyperlink ref="B7" r:id="rId6"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1511,64 +1450,64 @@
   <sheetData>
     <row r="1" spans="1:4" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A1" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="C1" s="12" t="s">
         <v>25</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="145.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B2" s="14">
         <v>0</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="14">
-        <v>150</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>30</v>
+        <v>2</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="90.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="18">
         <v>0</v>
       </c>
       <c r="C4" s="19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A5" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+    </row>
+    <row r="6" spans="1:4" ht="251.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A5" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-    </row>
-    <row r="6" spans="1:4" ht="251.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="26" t="s">
+      <c r="B6" s="29"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="15" t="s">
         <v>33</v>
-      </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="26"/>
-      <c r="D6" s="15" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>